<commit_message>
implement restoration monitoring logic
</commit_message>
<xml_diff>
--- a/data/Bioerosion_Data_EXAMPLE.xlsx
+++ b/data/Bioerosion_Data_EXAMPLE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B7C8E0-99B3-4A3A-8636-2B645D1DD653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0770CA7E-5685-4C6A-BFC1-42D29D7B042A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57495" yWindow="22140" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{19050643-5FB9-4299-B24C-C8F9EBB4329D}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="14566" windowHeight="7822" activeTab="1" xr2:uid="{19050643-5FB9-4299-B24C-C8F9EBB4329D}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="57">
   <si>
     <t>Taxon</t>
   </si>
@@ -185,9 +185,6 @@
   </si>
   <si>
     <t>Sparisoma aurofrenatum</t>
-  </si>
-  <si>
-    <t>20-90</t>
   </si>
   <si>
     <t>Scarus taeniopterus</t>
@@ -802,18 +799,18 @@
         <v>21</v>
       </c>
       <c r="G1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>30</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
         <v>31</v>
@@ -830,7 +827,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
         <v>30</v>
@@ -853,7 +850,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
         <v>30</v>
@@ -876,13 +873,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
         <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>33</v>
@@ -899,13 +896,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
@@ -922,16 +919,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
         <v>38</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" t="s">
-        <v>39</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -945,13 +942,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
@@ -968,13 +965,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="D9" t="s">
         <v>33</v>
@@ -991,13 +988,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
         <v>31</v>
@@ -1014,13 +1011,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
         <v>33</v>
@@ -1037,7 +1034,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
         <v>30</v>
@@ -1060,7 +1057,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
         <v>35</v>
@@ -1083,13 +1080,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
         <v>33</v>
@@ -1106,13 +1103,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
         <v>31</v>
@@ -1129,10 +1126,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>32</v>
@@ -1152,13 +1149,13 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
         <v>33</v>
@@ -1175,10 +1172,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>32</v>
@@ -1198,16 +1195,16 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" t="s">
         <v>38</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" t="s">
-        <v>39</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -1221,10 +1218,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>32</v>
@@ -1244,10 +1241,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>32</v>
@@ -1267,10 +1264,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>32</v>
@@ -1290,13 +1287,13 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
         <v>31</v>
@@ -1313,7 +1310,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
         <v>35</v>
@@ -1336,10 +1333,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>32</v>
@@ -1359,10 +1356,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>32</v>
@@ -1382,13 +1379,13 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D27" t="s">
         <v>33</v>
@@ -1405,10 +1402,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>32</v>
@@ -1428,13 +1425,13 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1451,13 +1448,13 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D30" t="s">
         <v>33</v>
@@ -1474,10 +1471,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>34</v>
@@ -1497,13 +1494,13 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" t="s">
         <v>35</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D32" t="s">
         <v>33</v>
@@ -1520,10 +1517,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>34</v>
@@ -1543,16 +1540,16 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B34" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D34" t="s">
         <v>38</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D34" t="s">
-        <v>39</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -1566,13 +1563,13 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D35" t="s">
         <v>31</v>
@@ -1589,10 +1586,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>34</v>
@@ -1657,18 +1654,18 @@
         <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
         <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>53</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1682,13 +1679,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
         <v>54</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1702,13 +1699,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
         <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>55</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1722,13 +1719,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1742,13 +1739,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
         <v>54</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -1798,15 +1795,15 @@
         <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2">
         <v>50</v>
@@ -1820,10 +1817,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3">
         <v>5</v>
@@ -1837,10 +1834,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1854,10 +1851,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -1871,10 +1868,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C6">
         <v>7</v>
@@ -1888,10 +1885,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7">
         <v>4</v>
@@ -1905,10 +1902,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -1922,10 +1919,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9">
         <v>4</v>
@@ -1939,10 +1936,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -1956,10 +1953,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -1973,10 +1970,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12">
         <v>6</v>

</xml_diff>